<commit_message>
Add Sep 17 3-handed session (+12.88)
</commit_message>
<xml_diff>
--- a/Poker Tracker.xlsx
+++ b/Poker Tracker.xlsx
@@ -888,28 +888,42 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
+      <c r="A6" s="3" t="n">
+        <v>46282</v>
+      </c>
       <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>PokerNow, 3-handed (online)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>112.88</v>
+      </c>
       <c r="F6" s="6">
         <f>IF(AND(D6="",E6=""),"",E6-D6)</f>
-        <v/>
+        <v>12.88</v>
       </c>
       <c r="G6" s="7" t="n"/>
-      <c r="H6" s="6">
+      <c r="H6" s="6" t="str">
         <f>IF(OR(G6="",G6=0,F6=""),"",F6/G6)</f>
         <v/>
       </c>
       <c r="I6" s="6">
         <f>IF(F6="","",IF(I5="",0,I5)+F6)</f>
-        <v/>
-      </c>
-      <c r="J6" s="4" t="n"/>
+        <v>64.57</v>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>vs tawer12 (+37.12) and vchen (-50.00). Stakes and hours not recorded.</t>
+        </is>
+      </c>
       <c r="K6" s="8">
         <f>IF(F6="",NA(),I6)</f>
-        <v/>
+        <v>64.57</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Add Sep 18 sessions: Poker at Berkeley (-22.64), heads-up vs Casey (+39.00), heads-up vs Aaron (-8.70)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Poker Tracker.xlsx
+++ b/Poker Tracker.xlsx
@@ -927,78 +927,136 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
+      <c r="A7" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>$0.25 / $0.50</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Poker at Berkeley (online)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>77.36</v>
+      </c>
       <c r="F7" s="6">
         <f>IF(AND(D7="",E7=""),"",E7-D7)</f>
-        <v/>
-      </c>
-      <c r="G7" s="7" t="n"/>
+        <v>-22.64</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>2</v>
+      </c>
       <c r="H7" s="6">
         <f>IF(OR(G7="",G7=0,F7=""),"",F7/G7)</f>
-        <v/>
+        <v>-11.32</v>
       </c>
       <c r="I7" s="6">
         <f>IF(F7="","",IF(I6="",0,I6)+F7)</f>
-        <v/>
-      </c>
-      <c r="J7" s="4" t="n"/>
+        <v>41.93</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Multiway. $100 total buy-in incl. 1 rebuy; cashed out $77.36.</t>
+        </is>
+      </c>
       <c r="K7" s="8">
         <f>IF(F7="",NA(),I7)</f>
-        <v/>
+        <v>41.93</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
+      <c r="A8" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>$0.25 / $0.50</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Heads-up, PokerNow (online)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>59</v>
+      </c>
       <c r="F8" s="6">
         <f>IF(AND(D8="",E8=""),"",E8-D8)</f>
-        <v/>
-      </c>
-      <c r="G8" s="7" t="n"/>
+        <v>39</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H8" s="6">
         <f>IF(OR(G8="",G8=0,F8=""),"",F8/G8)</f>
-        <v/>
+        <v>39.0</v>
       </c>
       <c r="I8" s="6">
         <f>IF(F8="","",IF(I7="",0,I7)+F8)</f>
-        <v/>
-      </c>
-      <c r="J8" s="4" t="n"/>
+        <v>80.93</v>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>vs Casey. Won $39 as reported; buy-in not given, assumed $20 (same as the Sep 17 heads-up).</t>
+        </is>
+      </c>
       <c r="K8" s="8">
         <f>IF(F8="",NA(),I8)</f>
-        <v/>
+        <v>80.93</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
+      <c r="A9" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>$0.10 / $0.20</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Heads-up, PokerNow (online)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>1.3</v>
+      </c>
       <c r="F9" s="6">
         <f>IF(AND(D9="",E9=""),"",E9-D9)</f>
-        <v/>
+        <v>-8.7</v>
       </c>
       <c r="G9" s="7" t="n"/>
-      <c r="H9" s="6">
+      <c r="H9" s="6" t="str">
         <f>IF(OR(G9="",G9=0,F9=""),"",F9/G9)</f>
         <v/>
       </c>
       <c r="I9" s="6">
         <f>IF(F9="","",IF(I8="",0,I8)+F9)</f>
-        <v/>
-      </c>
-      <c r="J9" s="4" t="n"/>
+        <v>72.23</v>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>vs Aaron. Bought in $10, cashed out $1.30. Hours not recorded.</t>
+        </is>
+      </c>
       <c r="K9" s="8">
         <f>IF(F9="",NA(),I9)</f>
-        <v/>
+        <v>72.23</v>
       </c>
     </row>
     <row r="10">
@@ -5865,7 +5923,7 @@
       </c>
       <c r="B4" s="13">
         <f>COUNT(Sessions!$D$2:$D$201)</f>
-        <v/>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -5876,7 +5934,7 @@
       </c>
       <c r="B5" s="14">
         <f>SUM(Sessions!$D$2:$D$201)</f>
-        <v/>
+        <v>420</v>
       </c>
     </row>
     <row r="6">
@@ -5887,7 +5945,7 @@
       </c>
       <c r="B6" s="14">
         <f>SUM(Sessions!$E$2:$E$201)</f>
-        <v/>
+        <v>492.23</v>
       </c>
     </row>
     <row r="7">
@@ -5898,7 +5956,7 @@
       </c>
       <c r="B7" s="14">
         <f>SUM(Sessions!$E$2:$E$201)-SUM(Sessions!$D$2:$D$201)</f>
-        <v/>
+        <v>72.23</v>
       </c>
     </row>
     <row r="8">
@@ -5909,7 +5967,7 @@
       </c>
       <c r="B8" s="15">
         <f>IF(SUM(Sessions!$D$2:$D$201)=0,"",(SUM(Sessions!$E$2:$E$201)-SUM(Sessions!$D$2:$D$201))/SUM(Sessions!$D$2:$D$201))</f>
-        <v/>
+        <v>0.171976</v>
       </c>
     </row>
     <row r="9">
@@ -5920,7 +5978,7 @@
       </c>
       <c r="B9" s="13">
         <f>COUNTIF(Sessions!$F$2:$F$201,"&gt;0")</f>
-        <v/>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -5931,7 +5989,7 @@
       </c>
       <c r="B10" s="13">
         <f>COUNTIF(Sessions!$F$2:$F$201,"&lt;0")</f>
-        <v/>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -5942,7 +6000,7 @@
       </c>
       <c r="B11" s="15">
         <f>IF(COUNT(Sessions!$D$2:$D$201)=0,"",COUNTIF(Sessions!$F$2:$F$201,"&gt;0")/COUNT(Sessions!$D$2:$D$201))</f>
-        <v/>
+        <v>0.625</v>
       </c>
     </row>
     <row r="12">
@@ -5953,7 +6011,7 @@
       </c>
       <c r="B12" s="14">
         <f>IF(COUNT(Sessions!$D$2:$D$201)=0,"",(SUM(Sessions!$E$2:$E$201)-SUM(Sessions!$D$2:$D$201))/COUNT(Sessions!$D$2:$D$201))</f>
-        <v/>
+        <v>9.0288</v>
       </c>
     </row>
     <row r="13">
@@ -5964,7 +6022,7 @@
       </c>
       <c r="B13" s="14">
         <f>IF(COUNT(Sessions!$D$2:$D$201)=0,"",MAX(Sessions!$F$2:$F$201))</f>
-        <v/>
+        <v>40.69</v>
       </c>
     </row>
     <row r="14">
@@ -5975,7 +6033,7 @@
       </c>
       <c r="B14" s="14">
         <f>IF(COUNT(Sessions!$D$2:$D$201)=0,"",MIN(Sessions!$F$2:$F$201))</f>
-        <v/>
+        <v>-40</v>
       </c>
     </row>
     <row r="15">
@@ -5986,7 +6044,7 @@
       </c>
       <c r="B15" s="16">
         <f>SUM(Sessions!$G$2:$G$201)</f>
-        <v/>
+        <v>5.5</v>
       </c>
     </row>
     <row r="16">
@@ -5997,7 +6055,7 @@
       </c>
       <c r="B16" s="14">
         <f>IF(SUM(Sessions!$G$2:$G$201)=0,"",SUMPRODUCT((Sessions!$G$2:$G$201&gt;0)*(Sessions!$F$2:$F$201))/SUM(Sessions!$G$2:$G$201))</f>
-        <v/>
+        <v>17.6455</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Add Sep 19 online session (+0.10)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Poker Tracker.xlsx
+++ b/Poker Tracker.xlsx
@@ -1060,28 +1060,44 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
+      <c r="A10" s="3" t="n">
+        <v>46284</v>
+      </c>
       <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Online (site not recorded)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>20.1</v>
+      </c>
       <c r="F10" s="6">
         <f>IF(AND(D10="",E10=""),"",E10-D10)</f>
-        <v/>
-      </c>
-      <c r="G10" s="7" t="n"/>
+        <v>0.1</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H10" s="6">
         <f>IF(OR(G10="",G10=0,F10=""),"",F10/G10)</f>
-        <v/>
+        <v>0.1</v>
       </c>
       <c r="I10" s="6">
         <f>IF(F10="","",IF(I9="",0,I9)+F10)</f>
-        <v/>
-      </c>
-      <c r="J10" s="4" t="n"/>
+        <v>72.33</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Bought in $20, cashed out $20.10. Stakes and site not recorded.</t>
+        </is>
+      </c>
       <c r="K10" s="8">
         <f>IF(F10="",NA(),I10)</f>
-        <v/>
+        <v>72.33</v>
       </c>
     </row>
     <row r="11">
@@ -5923,7 +5939,7 @@
       </c>
       <c r="B4" s="13">
         <f>COUNT(Sessions!$D$2:$D$201)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -5934,7 +5950,7 @@
       </c>
       <c r="B5" s="14">
         <f>SUM(Sessions!$D$2:$D$201)</f>
-        <v>420</v>
+        <v>440</v>
       </c>
     </row>
     <row r="6">
@@ -5945,7 +5961,7 @@
       </c>
       <c r="B6" s="14">
         <f>SUM(Sessions!$E$2:$E$201)</f>
-        <v>492.23</v>
+        <v>512.33</v>
       </c>
     </row>
     <row r="7">
@@ -5956,7 +5972,7 @@
       </c>
       <c r="B7" s="14">
         <f>SUM(Sessions!$E$2:$E$201)-SUM(Sessions!$D$2:$D$201)</f>
-        <v>72.23</v>
+        <v>72.33</v>
       </c>
     </row>
     <row r="8">
@@ -5967,7 +5983,7 @@
       </c>
       <c r="B8" s="15">
         <f>IF(SUM(Sessions!$D$2:$D$201)=0,"",(SUM(Sessions!$E$2:$E$201)-SUM(Sessions!$D$2:$D$201))/SUM(Sessions!$D$2:$D$201))</f>
-        <v>0.171976</v>
+        <v>0.164386</v>
       </c>
     </row>
     <row r="9">
@@ -5978,7 +5994,7 @@
       </c>
       <c r="B9" s="13">
         <f>COUNTIF(Sessions!$F$2:$F$201,"&gt;0")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -6000,7 +6016,7 @@
       </c>
       <c r="B11" s="15">
         <f>IF(COUNT(Sessions!$D$2:$D$201)=0,"",COUNTIF(Sessions!$F$2:$F$201,"&gt;0")/COUNT(Sessions!$D$2:$D$201))</f>
-        <v>0.625</v>
+        <v>0.666667</v>
       </c>
     </row>
     <row r="12">
@@ -6011,7 +6027,7 @@
       </c>
       <c r="B12" s="14">
         <f>IF(COUNT(Sessions!$D$2:$D$201)=0,"",(SUM(Sessions!$E$2:$E$201)-SUM(Sessions!$D$2:$D$201))/COUNT(Sessions!$D$2:$D$201))</f>
-        <v>9.0288</v>
+        <v>8.0367</v>
       </c>
     </row>
     <row r="13">
@@ -6044,7 +6060,7 @@
       </c>
       <c r="B15" s="16">
         <f>SUM(Sessions!$G$2:$G$201)</f>
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="16">
@@ -6055,7 +6071,7 @@
       </c>
       <c r="B16" s="14">
         <f>IF(SUM(Sessions!$G$2:$G$201)=0,"",SUMPRODUCT((Sessions!$G$2:$G$201&gt;0)*(Sessions!$F$2:$F$201))/SUM(Sessions!$G$2:$G$201))</f>
-        <v>17.6455</v>
+        <v>14.9462</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Add Sep 19 Poker at Berkeley session (-20)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Poker Tracker.xlsx
+++ b/Poker Tracker.xlsx
@@ -1101,28 +1101,44 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
+      <c r="A11" s="3" t="n">
+        <v>46284</v>
+      </c>
       <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Poker at Berkeley (Discord, online)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="F11" s="6">
         <f>IF(AND(D11="",E11=""),"",E11-D11)</f>
-        <v/>
-      </c>
-      <c r="G11" s="7" t="n"/>
+        <v>-20</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="H11" s="6">
         <f>IF(OR(G11="",G11=0,F11=""),"",F11/G11)</f>
-        <v/>
+        <v>-20</v>
       </c>
       <c r="I11" s="6">
         <f>IF(F11="","",IF(I10="",0,I10)+F11)</f>
-        <v/>
-      </c>
-      <c r="J11" s="4" t="n"/>
+        <v>52.33</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Lost the full $20 buy-in. Stakes not recorded.</t>
+        </is>
+      </c>
       <c r="K11" s="8">
         <f>IF(F11="",NA(),I11)</f>
-        <v/>
+        <v>52.33</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Add Sep 22 Poker at Berkeley session (-150)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Poker Tracker.xlsx
+++ b/Poker Tracker.xlsx
@@ -1142,28 +1142,42 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
+      <c r="A12" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>$0.25 / $0.50</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Poker at Berkeley (online)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="F12" s="6">
         <f>IF(AND(D12="",E12=""),"",E12-D12)</f>
-        <v/>
       </c>
       <c r="G12" s="7" t="n"/>
       <c r="H12" s="6">
         <f>IF(OR(G12="",G12=0,F12=""),"",F12/G12)</f>
-        <v/>
       </c>
       <c r="I12" s="6">
         <f>IF(F12="","",IF(I11="",0,I11)+F12)</f>
-        <v/>
-      </c>
-      <c r="J12" s="4" t="n"/>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Lost the full $150 buy-in. Hours not recorded.</t>
+        </is>
+      </c>
       <c r="K12" s="8">
         <f>IF(F12="",NA(),I12)</f>
-        <v/>
       </c>
     </row>
     <row r="13">

</xml_diff>